<commit_message>
Deepen Microfinance: loan loss provisioning, growth & officer productivity
Added days-past-due reserve tiering (Current/31-90/91-180/180+, standard
MFI provisioning bands) with required-vs-actual reserve adequacy check, and
a Growth & Productivity tab (borrower growth rate, loan-officer caseload,
disbursement per borrower).

Hand-verified provisioning math with a synthetic portfolio: tiers of
$10,000/$2,000/$500/$300 at 1%/10%/50%/100% -> required reserve $850 against
$12,800 outstanding; $800 actual reserve -> 94.12% adequacy. LibreOffice
recalc matched exactly.

11_Microfinance: 7 -> 18 formulas.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HRsbvuXZcdzPw9SqPDRRxr
</commit_message>
<xml_diff>
--- a/11_Microfinance/_template_MICROFINANCE.xlsx
+++ b/11_Microfinance/_template_MICROFINANCE.xlsx
@@ -11,7 +11,9 @@
     <sheet name="Cover" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Loan Portfolio" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Sustainability" sheetId="3" state="visible" r:id="rId5"/>
-    <sheet name="RefreshLog" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="Provisioning" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="Growth &amp; Productivity" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="RefreshLog" sheetId="6" state="visible" r:id="rId8"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -23,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="63">
   <si>
     <t xml:space="preserve">[MFI] — Microfinance Model</t>
   </si>
@@ -122,6 +124,78 @@
   </si>
   <si>
     <t xml:space="preserve">Portfolio yield (Rev / avg GLP)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Loan Loss Reserve Adequacy (days-past-due tiering)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aging bucket</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Outstanding balance ($)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reserve rate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Required reserve ($)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Current (0-30 days)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">31-90 days</t>
+  </si>
+  <si>
+    <t xml:space="preserve">91-180 days</t>
+  </si>
+  <si>
+    <t xml:space="preserve">180+ days / written off pending</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total outstanding portfolio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total required reserve (sum of tiers)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Actual reserve held ($)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reserve adequacy (actual / required)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;100% = under-reserved relative to portfolio risk profile — review provisioning policy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cross-check vs Loan Portfolio tab (should tie to GLP)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Growth &amp; Loan Officer Productivity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Active borrowers — prior period</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Active borrowers — current period</t>
+  </si>
+  <si>
+    <t xml:space="preserve">New disbursements this period ($)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Number of loan officers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Borrower growth rate (period over period)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Borrowers per loan officer (caseload)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Typical sustainable caseload benchmark: 250-400 borrowers/officer, group-lending-dependent</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Disbursement per active borrower ($, avg)</t>
   </si>
   <si>
     <t xml:space="preserve">Refresh Log</t>
@@ -152,7 +226,7 @@
     <numFmt numFmtId="166" formatCode="#,##0;\(#,##0\);\-"/>
     <numFmt numFmtId="167" formatCode="0.0%;\(0.0%\);\-"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -219,6 +293,13 @@
       <family val="0"/>
       <charset val="1"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF008000"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -295,7 +376,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="19">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -346,6 +427,26 @@
     </xf>
     <xf numFmtId="164" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
@@ -605,7 +706,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="B2:C7"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="30"/>
@@ -667,7 +768,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="B2:C16"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="30"/>
@@ -786,7 +887,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="B2:D14"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="34"/>
@@ -898,8 +999,263 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="B2:E14"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="40"/>
+  </cols>
+  <sheetData>
+    <row r="2" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B2" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B4" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="C4" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="D4" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="E4" s="12" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B5" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="C5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" s="13" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="E5" s="9" t="n">
+        <f aca="false">C5*D5</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B6" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="13" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E6" s="9" t="n">
+        <f aca="false">C6*D6</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B7" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="13" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E7" s="9" t="n">
+        <f aca="false">C7*D7</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B8" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="C8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" s="9" t="n">
+        <f aca="false">C8*D8</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B9" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C9" s="14" t="n">
+        <f aca="false">SUM(C5:C8)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B10" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="E10" s="14" t="n">
+        <f aca="false">SUM(E5:E8)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B12" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="C12" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B13" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="C13" s="15" t="str">
+        <f aca="false">IFERROR(C12/E10,"-")</f>
+        <v>-</v>
+      </c>
+      <c r="D13" s="11" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B14" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="C14" s="16" t="n">
+        <f aca="false">IFERROR(C9-'Loan Portfolio'!C5,"-")</f>
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="B2:D13"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="40"/>
+  </cols>
+  <sheetData>
+    <row r="2" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B2" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B4" s="7" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B5" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="C5" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B6" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="C6" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B7" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="C7" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B8" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C8" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B10" s="7" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B11" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="C11" s="8" t="str">
+        <f aca="false">IFERROR((C6-C5)/C5,"-")</f>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B12" s="0" t="s">
+        <v>54</v>
+      </c>
+      <c r="C12" s="17" t="str">
+        <f aca="false">IFERROR(C6/C8,"-")</f>
+        <v>-</v>
+      </c>
+      <c r="D12" s="11" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B13" s="0" t="s">
+        <v>56</v>
+      </c>
+      <c r="C13" s="9" t="str">
+        <f aca="false">IFERROR(C7/C6,"-")</f>
+        <v>-</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="B2:F14"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14"/>
@@ -910,95 +1266,95 @@
   <sheetData>
     <row r="2" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="1" t="s">
-        <v>33</v>
+        <v>57</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="12" t="s">
-        <v>34</v>
+        <v>58</v>
       </c>
       <c r="C4" s="12" t="s">
-        <v>35</v>
+        <v>59</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>36</v>
+        <v>60</v>
       </c>
       <c r="E4" s="12" t="s">
-        <v>37</v>
+        <v>61</v>
       </c>
       <c r="F4" s="12" t="s">
-        <v>38</v>
+        <v>62</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="13"/>
-      <c r="C5" s="13"/>
-      <c r="D5" s="13"/>
-      <c r="E5" s="13"/>
-      <c r="F5" s="13"/>
+      <c r="B5" s="18"/>
+      <c r="C5" s="18"/>
+      <c r="D5" s="18"/>
+      <c r="E5" s="18"/>
+      <c r="F5" s="18"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="13"/>
-      <c r="C6" s="13"/>
-      <c r="D6" s="13"/>
-      <c r="E6" s="13"/>
-      <c r="F6" s="13"/>
+      <c r="B6" s="18"/>
+      <c r="C6" s="18"/>
+      <c r="D6" s="18"/>
+      <c r="E6" s="18"/>
+      <c r="F6" s="18"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B7" s="13"/>
-      <c r="C7" s="13"/>
-      <c r="D7" s="13"/>
-      <c r="E7" s="13"/>
-      <c r="F7" s="13"/>
+      <c r="B7" s="18"/>
+      <c r="C7" s="18"/>
+      <c r="D7" s="18"/>
+      <c r="E7" s="18"/>
+      <c r="F7" s="18"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B8" s="13"/>
-      <c r="C8" s="13"/>
-      <c r="D8" s="13"/>
-      <c r="E8" s="13"/>
-      <c r="F8" s="13"/>
+      <c r="B8" s="18"/>
+      <c r="C8" s="18"/>
+      <c r="D8" s="18"/>
+      <c r="E8" s="18"/>
+      <c r="F8" s="18"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="13"/>
-      <c r="C9" s="13"/>
-      <c r="D9" s="13"/>
-      <c r="E9" s="13"/>
-      <c r="F9" s="13"/>
+      <c r="B9" s="18"/>
+      <c r="C9" s="18"/>
+      <c r="D9" s="18"/>
+      <c r="E9" s="18"/>
+      <c r="F9" s="18"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="13"/>
-      <c r="C10" s="13"/>
-      <c r="D10" s="13"/>
-      <c r="E10" s="13"/>
-      <c r="F10" s="13"/>
+      <c r="B10" s="18"/>
+      <c r="C10" s="18"/>
+      <c r="D10" s="18"/>
+      <c r="E10" s="18"/>
+      <c r="F10" s="18"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="13"/>
-      <c r="C11" s="13"/>
-      <c r="D11" s="13"/>
-      <c r="E11" s="13"/>
-      <c r="F11" s="13"/>
+      <c r="B11" s="18"/>
+      <c r="C11" s="18"/>
+      <c r="D11" s="18"/>
+      <c r="E11" s="18"/>
+      <c r="F11" s="18"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="13"/>
-      <c r="C12" s="13"/>
-      <c r="D12" s="13"/>
-      <c r="E12" s="13"/>
-      <c r="F12" s="13"/>
+      <c r="B12" s="18"/>
+      <c r="C12" s="18"/>
+      <c r="D12" s="18"/>
+      <c r="E12" s="18"/>
+      <c r="F12" s="18"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="13"/>
-      <c r="C13" s="13"/>
-      <c r="D13" s="13"/>
-      <c r="E13" s="13"/>
-      <c r="F13" s="13"/>
+      <c r="B13" s="18"/>
+      <c r="C13" s="18"/>
+      <c r="D13" s="18"/>
+      <c r="E13" s="18"/>
+      <c r="F13" s="18"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="13"/>
-      <c r="C14" s="13"/>
-      <c r="D14" s="13"/>
-      <c r="E14" s="13"/>
-      <c r="F14" s="13"/>
+      <c r="B14" s="18"/>
+      <c r="C14" s="18"/>
+      <c r="D14" s="18"/>
+      <c r="E14" s="18"/>
+      <c r="F14" s="18"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>